<commit_message>
MLB: add RL diagnostics and updated odds repricing
</commit_message>
<xml_diff>
--- a/mlb/predictions/April Predictions/April 21st/April 21st 2026 Predictions (Updated).xlsx
+++ b/mlb/predictions/April Predictions/April 21st/April 21st 2026 Predictions (Updated).xlsx
@@ -66,12 +66,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00EAF8F1"/>
+        <fgColor rgb="00FFF1EC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF1EC"/>
+        <fgColor rgb="00EAF8F1"/>
       </patternFill>
     </fill>
   </fills>
@@ -606,20 +606,18 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>HOU Moneyline</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>2.25</v>
-      </c>
+          <t>SKIP - Missing odds data</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n"/>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>EUR 16.93</t>
+          <t>EUR 0.00</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>BET</t>
+          <t>SKIP</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr"/>
@@ -634,278 +632,278 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>Cincinnati Reds vs Tampa Bay Rays (Game 2 of 3)</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>CIN Moneyline</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="n">
-        <v>1.87</v>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>CIN -2.5 (Run Line)</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>EUR 5.64</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="7" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr"/>
-      <c r="G8" s="6">
+      <c r="F8" s="7" t="inlineStr"/>
+      <c r="G8" s="9">
         <f>IF(E8&lt;&gt;"BET",0,IF(F8="Win",(C8-1)*VALUE(SUBSTITUTE(D8,"EUR ","")),IF(F8="Loss",-VALUE(SUBSTITUTE(D8,"EUR ","")),IF(F8="Push",0,""))))</f>
         <v/>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="7" t="inlineStr">
         <is>
           <t>822995</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>St. Louis Cardinals vs Miami Marlins (Game 2 of 3)</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>MIA Moneyline</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>1.83</v>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>EUR 2.82</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>MIA -1.5 (Run Line)</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>2.71</v>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>EUR 5.64</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr"/>
-      <c r="G9" s="6">
+      <c r="F9" s="7" t="inlineStr"/>
+      <c r="G9" s="9">
         <f>IF(E9&lt;&gt;"BET",0,IF(F9="Win",(C9-1)*VALUE(SUBSTITUTE(D9,"EUR ","")),IF(F9="Loss",-VALUE(SUBSTITUTE(D9,"EUR ","")),IF(F9="Push",0,""))))</f>
         <v/>
       </c>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>823880</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Milwaukee Brewers vs Detroit Tigers (Game 1 of 3)</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>MIL Moneyline</t>
         </is>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="8" t="n">
         <v>1.91</v>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>EUR 16.93</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr"/>
-      <c r="G10" s="6">
+      <c r="F10" s="7" t="inlineStr"/>
+      <c r="G10" s="9">
         <f>IF(E10&lt;&gt;"BET",0,IF(F10="Win",(C10-1)*VALUE(SUBSTITUTE(D10,"EUR ","")),IF(F10="Loss",-VALUE(SUBSTITUTE(D10,"EUR ","")),IF(F10="Push",0,""))))</f>
         <v/>
       </c>
-      <c r="H10" s="4" t="inlineStr">
+      <c r="H10" s="7" t="inlineStr">
         <is>
           <t>824290</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Atlanta Braves vs Washington Nationals (Game 2 of 4)</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>SKIP - Missing odds data</t>
         </is>
       </c>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>EUR 0.00</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="4" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr"/>
-      <c r="G11" s="9">
+      <c r="F11" s="4" t="inlineStr"/>
+      <c r="G11" s="6">
         <f>IF(E11&lt;&gt;"BET",0,IF(F11="Win",(C11-1)*VALUE(SUBSTITUTE(D11,"EUR ","")),IF(F11="Loss",-VALUE(SUBSTITUTE(D11,"EUR ","")),IF(F11="Push",0,""))))</f>
         <v/>
       </c>
-      <c r="H11" s="7" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr">
         <is>
           <t>822747</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>New York Yankees vs Boston Red Sox (Game 1 of 3)</t>
         </is>
       </c>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>NYY Moneyline</t>
         </is>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>EUR 16.93</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr"/>
-      <c r="G12" s="6">
+      <c r="F12" s="7" t="inlineStr"/>
+      <c r="G12" s="9">
         <f>IF(E12&lt;&gt;"BET",0,IF(F12="Win",(C12-1)*VALUE(SUBSTITUTE(D12,"EUR ","")),IF(F12="Loss",-VALUE(SUBSTITUTE(D12,"EUR ","")),IF(F12="Push",0,""))))</f>
         <v/>
       </c>
-      <c r="H12" s="4" t="inlineStr">
+      <c r="H12" s="7" t="inlineStr">
         <is>
           <t>824773</t>
         </is>
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>Minnesota Twins vs New York Mets (Game 1 of 3)</t>
         </is>
       </c>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>MIN Moneyline</t>
         </is>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="8" t="n">
         <v>2.3</v>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>EUR 22.57</t>
         </is>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr"/>
-      <c r="G13" s="6">
+      <c r="F13" s="7" t="inlineStr"/>
+      <c r="G13" s="9">
         <f>IF(E13&lt;&gt;"BET",0,IF(F13="Win",(C13-1)*VALUE(SUBSTITUTE(D13,"EUR ","")),IF(F13="Loss",-VALUE(SUBSTITUTE(D13,"EUR ","")),IF(F13="Push",0,""))))</f>
         <v/>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>823640</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Baltimore Orioles vs Kansas City Royals (Game 2 of 3)</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>BAL Moneyline</t>
         </is>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C14" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>EUR 11.28</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" s="7" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr"/>
-      <c r="G14" s="6">
+      <c r="F14" s="7" t="inlineStr"/>
+      <c r="G14" s="9">
         <f>IF(E14&lt;&gt;"BET",0,IF(F14="Win",(C14-1)*VALUE(SUBSTITUTE(D14,"EUR ","")),IF(F14="Loss",-VALUE(SUBSTITUTE(D14,"EUR ","")),IF(F14="Push",0,""))))</f>
         <v/>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="7" t="inlineStr">
         <is>
           <t>824127</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>Philadelphia Phillies vs Chicago Cubs (Game 2 of 4)</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>PHI Moneyline</t>
         </is>
       </c>
-      <c r="C15" s="5" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>EUR 22.57</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="C15" s="8" t="n">
+        <v>2.05</v>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>EUR 16.93</t>
+        </is>
+      </c>
+      <c r="E15" s="7" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr"/>
-      <c r="G15" s="6">
+      <c r="F15" s="7" t="inlineStr"/>
+      <c r="G15" s="9">
         <f>IF(E15&lt;&gt;"BET",0,IF(F15="Win",(C15-1)*VALUE(SUBSTITUTE(D15,"EUR ","")),IF(F15="Loss",-VALUE(SUBSTITUTE(D15,"EUR ","")),IF(F15="Push",0,""))))</f>
         <v/>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>824690</t>
         </is>
@@ -919,20 +917,20 @@
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>SKIP - SP not yet announced</t>
+          <t>PIT Moneyline</t>
         </is>
       </c>
       <c r="C16" s="8" t="n">
-        <v>1.91</v>
+        <v>1.95</v>
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>EUR 2.82</t>
+          <t>EUR 5.64</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>SKIP</t>
+          <t>BET</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr"/>
@@ -947,175 +945,175 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>San Diego Padres vs Colorado Rockies (Game 1 of 3)</t>
         </is>
       </c>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>SD Moneyline</t>
         </is>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C17" s="8" t="n">
         <v>1.67</v>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>EUR 11.28</t>
         </is>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr"/>
-      <c r="G17" s="6">
+      <c r="F17" s="7" t="inlineStr"/>
+      <c r="G17" s="9">
         <f>IF(E17&lt;&gt;"BET",0,IF(F17="Win",(C17-1)*VALUE(SUBSTITUTE(D17,"EUR ","")),IF(F17="Loss",-VALUE(SUBSTITUTE(D17,"EUR ","")),IF(F17="Push",0,""))))</f>
         <v/>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>824369</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="4" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>Toronto Blue Jays vs Los Angeles Angels (Game 2 of 3)</t>
         </is>
       </c>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>TOR Moneyline</t>
         </is>
       </c>
-      <c r="C18" s="5" t="n">
+      <c r="C18" s="8" t="n">
         <v>1.91</v>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>EUR 16.93</t>
         </is>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" s="7" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr"/>
-      <c r="G18" s="6">
+      <c r="F18" s="7" t="inlineStr"/>
+      <c r="G18" s="9">
         <f>IF(E18&lt;&gt;"BET",0,IF(F18="Win",(C18-1)*VALUE(SUBSTITUTE(D18,"EUR ","")),IF(F18="Loss",-VALUE(SUBSTITUTE(D18,"EUR ","")),IF(F18="Push",0,""))))</f>
         <v/>
       </c>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H18" s="7" t="inlineStr">
         <is>
           <t>824045</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="4" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>Athletics vs Seattle Mariners (Game 2 of 3)</t>
         </is>
       </c>
-      <c r="B19" s="4" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>ATH Moneyline</t>
         </is>
       </c>
-      <c r="C19" s="5" t="n">
+      <c r="C19" s="8" t="n">
         <v>2.38</v>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>EUR 22.57</t>
         </is>
       </c>
-      <c r="E19" s="4" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F19" s="4" t="inlineStr"/>
-      <c r="G19" s="6">
+      <c r="F19" s="7" t="inlineStr"/>
+      <c r="G19" s="9">
         <f>IF(E19&lt;&gt;"BET",0,IF(F19="Win",(C19-1)*VALUE(SUBSTITUTE(D19,"EUR ","")),IF(F19="Loss",-VALUE(SUBSTITUTE(D19,"EUR ","")),IF(F19="Push",0,""))))</f>
         <v/>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>823148</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Chicago White Sox vs Arizona Diamondbacks (Game 1 of 3)</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B20" s="4" t="inlineStr">
         <is>
           <t>SKIP - No clear edge</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n">
+      <c r="C20" s="5" t="n">
         <v>1.65</v>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>EUR 0.00</t>
         </is>
       </c>
-      <c r="E20" s="7" t="inlineStr">
+      <c r="E20" s="4" t="inlineStr">
         <is>
           <t>SKIP</t>
         </is>
       </c>
-      <c r="F20" s="7" t="inlineStr"/>
-      <c r="G20" s="9">
+      <c r="F20" s="4" t="inlineStr"/>
+      <c r="G20" s="6">
         <f>IF(E20&lt;&gt;"BET",0,IF(F20="Win",(C20-1)*VALUE(SUBSTITUTE(D20,"EUR ","")),IF(F20="Loss",-VALUE(SUBSTITUTE(D20,"EUR ","")),IF(F20="Push",0,""))))</f>
         <v/>
       </c>
-      <c r="H20" s="7" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>825099</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers vs San Francisco Giants (Game 1 of 3)</t>
         </is>
       </c>
-      <c r="B21" s="4" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>LAD Moneyline</t>
         </is>
       </c>
-      <c r="C21" s="5" t="n">
+      <c r="C21" s="8" t="n">
         <v>1.53</v>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>EUR 5.64</t>
         </is>
       </c>
-      <c r="E21" s="4" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F21" s="4" t="inlineStr"/>
-      <c r="G21" s="6">
+      <c r="F21" s="7" t="inlineStr"/>
+      <c r="G21" s="9">
         <f>IF(E21&lt;&gt;"BET",0,IF(F21="Win",(C21-1)*VALUE(SUBSTITUTE(D21,"EUR ","")),IF(F21="Loss",-VALUE(SUBSTITUTE(D21,"EUR ","")),IF(F21="Push",0,""))))</f>
         <v/>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>823236</t>
         </is>

</xml_diff>

<commit_message>
MMA: ledger-first architecture refactor (Phase 1–5)
- ledger.py: SQLite financial core v5 with append-only ledger, hash chain,
  pipeline locking, FK repair on startup, edge/confidence/acca_legs columns
- app.py: load_staking() reads ONLY from ledger.db (no staking_plan.json);
  enrich_fight() strips Pass/Avoid/unpriced markets before templates see them;
  get_event_bets() provides ledger-native bet data with reshaping for templates
- betting_model.py: stamps deterministic bet_id on each single; place_bets()
  stores edge, confidence, acca_legs_json per bet
- fetch_card.py: date-based auto-selection of next upcoming UFC event (removes
  hardcoded TARGET_KEYWORDS that caused wrong card to be fetched)
- bankroll.py: current_bankroll() delegates to ledger.current_bankroll_from_db()
- New: backup.py, integrity.py, scheduler.py, auth.py, settle/history templates

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mlb/predictions/April Predictions/April 21st/April 21st 2026 Predictions (Updated).xlsx
+++ b/mlb/predictions/April Predictions/April 21st/April 21st 2026 Predictions (Updated).xlsx
@@ -42,7 +42,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -74,6 +74,16 @@
         <fgColor rgb="00EAF8F1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -101,7 +111,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -133,6 +143,24 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -632,31 +660,35 @@
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="13" t="inlineStr">
         <is>
           <t>Cincinnati Reds vs Tampa Bay Rays (Game 2 of 3)</t>
         </is>
       </c>
-      <c r="B8" s="7" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>CIN -2.5 (Run Line)</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="14" t="n">
         <v>3.4</v>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>EUR 5.64</t>
         </is>
       </c>
-      <c r="E8" s="7" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F8" s="7" t="inlineStr"/>
-      <c r="G8" s="9">
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="G8" s="15">
         <f>IF(E8&lt;&gt;"BET",0,IF(F8="Win",(C8-1)*VALUE(SUBSTITUTE(D8,"EUR ","")),IF(F8="Loss",-VALUE(SUBSTITUTE(D8,"EUR ","")),IF(F8="Push",0,""))))</f>
         <v/>
       </c>
@@ -667,31 +699,35 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>St. Louis Cardinals vs Miami Marlins (Game 2 of 3)</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>MIA -1.5 (Run Line)</t>
         </is>
       </c>
-      <c r="C9" s="8" t="n">
+      <c r="C9" s="17" t="n">
         <v>2.71</v>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>EUR 5.64</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr"/>
-      <c r="G9" s="9">
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="G9" s="18">
         <f>IF(E9&lt;&gt;"BET",0,IF(F9="Win",(C9-1)*VALUE(SUBSTITUTE(D9,"EUR ","")),IF(F9="Loss",-VALUE(SUBSTITUTE(D9,"EUR ","")),IF(F9="Push",0,""))))</f>
         <v/>
       </c>
@@ -702,31 +738,35 @@
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="13" t="inlineStr">
         <is>
           <t>Milwaukee Brewers vs Detroit Tigers (Game 1 of 3)</t>
         </is>
       </c>
-      <c r="B10" s="7" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>MIL Moneyline</t>
         </is>
       </c>
-      <c r="C10" s="8" t="n">
+      <c r="C10" s="14" t="n">
         <v>1.91</v>
       </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>EUR 16.93</t>
         </is>
       </c>
-      <c r="E10" s="7" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F10" s="7" t="inlineStr"/>
-      <c r="G10" s="9">
+      <c r="F10" s="13" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="G10" s="15">
         <f>IF(E10&lt;&gt;"BET",0,IF(F10="Win",(C10-1)*VALUE(SUBSTITUTE(D10,"EUR ","")),IF(F10="Loss",-VALUE(SUBSTITUTE(D10,"EUR ","")),IF(F10="Push",0,""))))</f>
         <v/>
       </c>
@@ -770,31 +810,35 @@
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
-      <c r="A12" s="7" t="inlineStr">
+      <c r="A12" s="13" t="inlineStr">
         <is>
           <t>New York Yankees vs Boston Red Sox (Game 1 of 3)</t>
         </is>
       </c>
-      <c r="B12" s="7" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>NYY Moneyline</t>
         </is>
       </c>
-      <c r="C12" s="8" t="n">
+      <c r="C12" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="7" t="inlineStr">
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>EUR 16.93</t>
         </is>
       </c>
-      <c r="E12" s="7" t="inlineStr">
+      <c r="E12" s="13" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F12" s="7" t="inlineStr"/>
-      <c r="G12" s="9">
+      <c r="F12" s="13" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="G12" s="15">
         <f>IF(E12&lt;&gt;"BET",0,IF(F12="Win",(C12-1)*VALUE(SUBSTITUTE(D12,"EUR ","")),IF(F12="Loss",-VALUE(SUBSTITUTE(D12,"EUR ","")),IF(F12="Push",0,""))))</f>
         <v/>
       </c>
@@ -805,31 +849,35 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1">
-      <c r="A13" s="7" t="inlineStr">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>Minnesota Twins vs New York Mets (Game 1 of 3)</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>MIN Moneyline</t>
         </is>
       </c>
-      <c r="C13" s="8" t="n">
+      <c r="C13" s="14" t="n">
         <v>2.3</v>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>EUR 22.57</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E13" s="13" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr"/>
-      <c r="G13" s="9">
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="G13" s="15">
         <f>IF(E13&lt;&gt;"BET",0,IF(F13="Win",(C13-1)*VALUE(SUBSTITUTE(D13,"EUR ","")),IF(F13="Loss",-VALUE(SUBSTITUTE(D13,"EUR ","")),IF(F13="Push",0,""))))</f>
         <v/>
       </c>
@@ -840,31 +888,35 @@
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Baltimore Orioles vs Kansas City Royals (Game 2 of 3)</t>
         </is>
       </c>
-      <c r="B14" s="7" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>BAL Moneyline</t>
         </is>
       </c>
-      <c r="C14" s="8" t="n">
+      <c r="C14" s="17" t="n">
         <v>2</v>
       </c>
-      <c r="D14" s="7" t="inlineStr">
+      <c r="D14" s="16" t="inlineStr">
         <is>
           <t>EUR 11.28</t>
         </is>
       </c>
-      <c r="E14" s="7" t="inlineStr">
+      <c r="E14" s="16" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F14" s="7" t="inlineStr"/>
-      <c r="G14" s="9">
+      <c r="F14" s="16" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="G14" s="18">
         <f>IF(E14&lt;&gt;"BET",0,IF(F14="Win",(C14-1)*VALUE(SUBSTITUTE(D14,"EUR ","")),IF(F14="Loss",-VALUE(SUBSTITUTE(D14,"EUR ","")),IF(F14="Push",0,""))))</f>
         <v/>
       </c>
@@ -875,31 +927,35 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Philadelphia Phillies vs Chicago Cubs (Game 2 of 4)</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>PHI Moneyline</t>
         </is>
       </c>
-      <c r="C15" s="8" t="n">
+      <c r="C15" s="17" t="n">
         <v>2.05</v>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="16" t="inlineStr">
         <is>
           <t>EUR 16.93</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="16" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr"/>
-      <c r="G15" s="9">
+      <c r="F15" s="16" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="G15" s="18">
         <f>IF(E15&lt;&gt;"BET",0,IF(F15="Win",(C15-1)*VALUE(SUBSTITUTE(D15,"EUR ","")),IF(F15="Loss",-VALUE(SUBSTITUTE(D15,"EUR ","")),IF(F15="Push",0,""))))</f>
         <v/>
       </c>
@@ -910,31 +966,35 @@
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="7" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>Pittsburgh Pirates vs Texas Rangers (Game 1 of 3)</t>
         </is>
       </c>
-      <c r="B16" s="7" t="inlineStr">
+      <c r="B16" s="16" t="inlineStr">
         <is>
           <t>PIT Moneyline</t>
         </is>
       </c>
-      <c r="C16" s="8" t="n">
+      <c r="C16" s="17" t="n">
         <v>1.95</v>
       </c>
-      <c r="D16" s="7" t="inlineStr">
+      <c r="D16" s="16" t="inlineStr">
         <is>
           <t>EUR 5.64</t>
         </is>
       </c>
-      <c r="E16" s="7" t="inlineStr">
+      <c r="E16" s="16" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F16" s="7" t="inlineStr"/>
-      <c r="G16" s="9">
+      <c r="F16" s="16" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="G16" s="18">
         <f>IF(E16&lt;&gt;"BET",0,IF(F16="Win",(C16-1)*VALUE(SUBSTITUTE(D16,"EUR ","")),IF(F16="Loss",-VALUE(SUBSTITUTE(D16,"EUR ","")),IF(F16="Push",0,""))))</f>
         <v/>
       </c>
@@ -945,31 +1005,35 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>San Diego Padres vs Colorado Rockies (Game 1 of 3)</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>SD Moneyline</t>
         </is>
       </c>
-      <c r="C17" s="8" t="n">
+      <c r="C17" s="14" t="n">
         <v>1.67</v>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>EUR 11.28</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E17" s="13" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr"/>
-      <c r="G17" s="9">
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="G17" s="15">
         <f>IF(E17&lt;&gt;"BET",0,IF(F17="Win",(C17-1)*VALUE(SUBSTITUTE(D17,"EUR ","")),IF(F17="Loss",-VALUE(SUBSTITUTE(D17,"EUR ","")),IF(F17="Push",0,""))))</f>
         <v/>
       </c>
@@ -980,31 +1044,35 @@
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
-      <c r="A18" s="7" t="inlineStr">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>Toronto Blue Jays vs Los Angeles Angels (Game 2 of 3)</t>
         </is>
       </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>TOR Moneyline</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n">
+      <c r="C18" s="14" t="n">
         <v>1.91</v>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="13" t="inlineStr">
         <is>
           <t>EUR 16.93</t>
         </is>
       </c>
-      <c r="E18" s="7" t="inlineStr">
+      <c r="E18" s="13" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F18" s="7" t="inlineStr"/>
-      <c r="G18" s="9">
+      <c r="F18" s="13" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="G18" s="15">
         <f>IF(E18&lt;&gt;"BET",0,IF(F18="Win",(C18-1)*VALUE(SUBSTITUTE(D18,"EUR ","")),IF(F18="Loss",-VALUE(SUBSTITUTE(D18,"EUR ","")),IF(F18="Push",0,""))))</f>
         <v/>
       </c>
@@ -1015,31 +1083,35 @@
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>Athletics vs Seattle Mariners (Game 2 of 3)</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>ATH Moneyline</t>
         </is>
       </c>
-      <c r="C19" s="8" t="n">
+      <c r="C19" s="14" t="n">
         <v>2.38</v>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="13" t="inlineStr">
         <is>
           <t>EUR 22.57</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E19" s="13" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr"/>
-      <c r="G19" s="9">
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
+      <c r="G19" s="15">
         <f>IF(E19&lt;&gt;"BET",0,IF(F19="Win",(C19-1)*VALUE(SUBSTITUTE(D19,"EUR ","")),IF(F19="Loss",-VALUE(SUBSTITUTE(D19,"EUR ","")),IF(F19="Push",0,""))))</f>
         <v/>
       </c>
@@ -1085,31 +1157,35 @@
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="7" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>Los Angeles Dodgers vs San Francisco Giants (Game 1 of 3)</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
         <is>
           <t>LAD Moneyline</t>
         </is>
       </c>
-      <c r="C21" s="8" t="n">
+      <c r="C21" s="17" t="n">
         <v>1.53</v>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D21" s="16" t="inlineStr">
         <is>
           <t>EUR 5.64</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E21" s="16" t="inlineStr">
         <is>
           <t>BET</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr"/>
-      <c r="G21" s="9">
+      <c r="F21" s="16" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
+      <c r="G21" s="18">
         <f>IF(E21&lt;&gt;"BET",0,IF(F21="Win",(C21-1)*VALUE(SUBSTITUTE(D21,"EUR ","")),IF(F21="Loss",-VALUE(SUBSTITUTE(D21,"EUR ","")),IF(F21="Push",0,""))))</f>
         <v/>
       </c>
@@ -1119,6 +1195,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="10" t="inlineStr">
         <is>

</xml_diff>